<commit_message>
Campagne de groupe, bugs 11-12, tests utilisateurs et preuves
- Ajout des 17 cas de test de Marina (navigateur + Swagger), 44 cas au total
- BUG-11 (minimum de commande ignoré) et BUG-12 (favoris impossibles)
- Captures d'écran dans docs/preuves (navigateur, Swagger, DevTools)
- Tests utilisateurs : 2 participantes, 3 scénarios (user-feedback.md)
- Mise à jour du rapport, de la matrice de risques et du plan d'amélioration

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -488,6 +488,8 @@
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -546,6 +548,16 @@
           <t>Bug lié</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Testé par</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Preuve</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -599,6 +611,16 @@
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -652,6 +674,16 @@
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -705,6 +737,16 @@
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -759,6 +801,16 @@
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -816,6 +868,16 @@
           <t>BUG-02</t>
         </is>
       </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>BUG-02 (réponse HTML)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -869,6 +931,16 @@
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -922,6 +994,16 @@
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -975,6 +1057,16 @@
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1028,6 +1120,16 @@
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1081,6 +1183,16 @@
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1134,6 +1246,16 @@
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1187,6 +1309,16 @@
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1240,6 +1372,16 @@
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1293,6 +1435,16 @@
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>preuves/ui-mot-de-passe-trop-court.png</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1350,6 +1502,16 @@
           <t>BUG-06</t>
         </is>
       </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>BUG-06 (réponse API)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1407,6 +1569,16 @@
           <t>BUG-07</t>
         </is>
       </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>BUG-07 (réponse API)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1464,6 +1636,16 @@
           <t>BUG-04</t>
         </is>
       </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>BUG-04 (réponse API)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1517,6 +1699,16 @@
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1571,6 +1763,16 @@
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1624,6 +1826,16 @@
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1677,6 +1889,16 @@
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Réponse API / HTML notée dans « Résultat obtenu »</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1732,6 +1954,16 @@
       <c r="K23" s="5" t="inlineStr">
         <is>
           <t>BUG-01</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>BUG-01 + preuves/swagger-coupon-atlas15-10pourcent.png</t>
         </is>
       </c>
     </row>
@@ -1793,6 +2025,16 @@
           <t>BUG-03</t>
         </is>
       </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>BUG-03 (séquence API)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1852,6 +2094,16 @@
           <t>BUG-05</t>
         </is>
       </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>BUG-05 (compteurs avant/après)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1909,6 +2161,16 @@
           <t>BUG-09</t>
         </is>
       </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>BUG-09 (requête SQL)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1964,6 +2226,16 @@
       <c r="K27" s="5" t="inlineStr">
         <is>
           <t>BUG-08</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>BUG-08 (séquence admin)</t>
         </is>
       </c>
     </row>
@@ -2023,6 +2295,1143 @@
       <c r="K28" s="5" t="inlineStr">
         <is>
           <t>BUG-10</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Elodie</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>BUG-10 (requête SQL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC-M01</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Connexion avec identifiants valides</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'un utilisateur enregistré peut se connecter</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Compte alice@example.com existant, utilisateur déconnecté</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>alice@example.com / Password123!</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>1. Ouvrir /login
+2. Saisir email et mot de passe
+3. Cliquer sur « Se connecter »</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Redirection vers l'accueil, utilisateur connecté</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Accueil affiché, « Alice Martin » visible dans la barre du haut</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>preuves/ui-connexion-ok.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-M02</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Création d'un compte avec données valides</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'un nouvel utilisateur peut créer un compte</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Email non encore utilisé</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Test User / testuser01@example.com / TestPass123!</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>1. Ouvrir « Créer un compte »
+2. Saisir nom, email, mot de passe
+3. Cliquer sur « Créer mon compte »</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Compte créé, utilisateur connecté</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Redirection vers l'accueil avec le nom affiché dans la barre du haut</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Navigateur (constat visuel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-M03</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Filtre par catégorie (Japonais)</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier que le filtre catégorie affine la liste des restaurants</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>category=Japonais</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>1. Accueil &gt; « Toutes les catégories » &gt; Japonais
+2. Cliquer sur « Rechercher »
+3. Rejouer GET /api/restaurants?category=Japonais dans Swagger</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Seuls les restaurants japonais sont affichés</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Tokyo Bowl et Night Sushi uniquement (count = 2)</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>preuves/swagger-filtre-categorie-japonais.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-M04</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Commande complète depuis l'interface</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier le parcours ajout &gt; panier &gt; checkout &gt; confirmation</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Utilisateur connecté, produit en stock</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Chicken Teriyaki x1</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>1. Ajouter le produit
+2. Ouvrir le panier, vérifier le total
+3. Passer commande
+4. Confirmer</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Commande validée, message de confirmation, panier vidé</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Commande confirmée, panier vide</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Navigateur (constat visuel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-M05</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Erreur</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Ajout d'un restaurant aux favoris</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'on peut ajouter un restaurant aux favoris et le retrouver dans le profil</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Utilisateur connecté</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Restaurant Green Kitchen / Tokyo Bowl</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>1. Ouvrir la fiche d'un restaurant
+2. Chercher un bouton « favori »
+3. Ouvrir Mon profil &gt; Favoris</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Un bouton permet d'ajouter le restaurant, qui apparaît ensuite dans « Favoris »</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Aucun bouton favori sur les pages ; la section « Favoris » du profil reste « Aucun favori. »</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>BUG-12</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>preuves/ui-pas-de-bouton-favori.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-M06</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Erreur</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Création de compte avec un email déjà utilisé</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier le refus d'un email déjà enregistré</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Compte alice@example.com existant</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Alice Bis / alice@example.com / Nouveau123!</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>1. Ouvrir « Créer un compte »
+2. Saisir l'email existant
+3. Valider</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Message d'erreur, aucun compte créé</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>« Un compte existe déjà avec cet email. », aucun compte créé</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>preuves/ui-email-deja-utilise.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-M07</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Erreur</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Création de compte avec champs vides</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier que le formulaire bloque les champs obligatoires vides</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Page « Créer un compte » ouverte</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Tous les champs vides</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>1. Laisser les champs vides
+2. Cliquer sur « Créer mon compte »</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Formulaire non soumis, message d'erreur</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>« Veuillez renseigner ce champ », aucun compte créé</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr"/>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>Navigateur (constat visuel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-M08</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Erreur</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Ajout au panier d'un produit HORS STOCK (interface)</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'un produit affiché « HORS STOCK » ne peut pas être ajouté</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Tokyo Bowl : Salmon Bowl / Gyozas affichés « HORS STOCK »</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Quantité 1</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>1. Ouvrir le menu de Tokyo Bowl
+2. Cliquer sur « Ajouter » sous un produit HORS STOCK</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Bouton « Ajouter » désactivé</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Bouton actif : « Salmon Bowl ajouté au panier. », stock affiché ensuite à -2</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>BUG-07</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>preuves/ui-hors-stock-ajoute-au-panier.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC-M09</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Erreur</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Checkout avec un panier vide</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'on ne peut pas valider une commande sans produit</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Utilisateur connecté, panier vide</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>1. Ouvrir la page « Panier »
+2. Chercher un moyen de valider</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Aucun bouton de validation</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Aucun bouton « Passer commande » affiché</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr"/>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>Navigateur (constat visuel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TC-M10</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Limite</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Mot de passe à la longueur minimale (8)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'un mot de passe de exactement 8 caractères est accepté</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Page « Créer un compte » ouverte</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>testlimite@example.com / Abcd123! (8 caractères)</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>1. Saisir nom, email et un mot de passe de 8 caractères
+2. Valider</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Compte créé</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Compte créé</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Navigateur (constat visuel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TC-M11</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Limite</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Quantité égale au stock restant</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'on peut commander exactement le stock disponible</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Salmon Bowl : stock 2</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Quantité 2</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>1. Menu Tokyo Bowl
+2. Quantité 2 sur Salmon Bowl
+3. Ajouter puis commander</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Ajout et commande acceptés, stock à 0</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Ajout accepté, le produit passe ensuite en rupture</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>Navigateur (constat visuel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TC-M12</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Limite</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Quantité supérieure au stock (stock 0)</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier le refus d'une quantité supérieure au stock</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Salmon Bowl : stock 0</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Quantité 3</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>1. Menu Tokyo Bowl
+2. Quantité 3 sur Salmon Bowl
+3. Ajouter puis commander
+4. Vérifier le stock dans Swagger (GET /api/restaurants/2/products)</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Ajout refusé, rien dans le panier</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Ajout et commande acceptés, stock à -2</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>BUG-07</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>preuves/swagger-salmon-bowl-stock-negatif.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>TC-M13</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Limite</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Quantité au-delà du stock dans le panier (99 pour 98)</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier que la quantité du panier est plafonnée au stock</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Produit avec stock 98</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Quantité 99</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>1. Ajouter le produit
+2. Mettre 99 dans le panier
+3. Mettre à jour puis passer commande</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Quantité refusée ou plafonnée à 98</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>99 acceptés (346,50 €), commande validée</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>BUG-07</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>preuves/ui-panier-quantite-99.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TC-M14</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Règle métier</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Le stock diminue après commande</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier que commander décrémente le stock</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Tofu Bowl : stock 100</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Quantité 1</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>1. Noter le stock
+2. Commander 1 unité
+3. Revenir au menu</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Stock passe de 100 à 99</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Stock à 99</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr"/>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>Navigateur (constat visuel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>TC-M15</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Règle métier</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Minimum de commande du restaurant</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'une commande sous le minimum du restaurant est refusée</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Burger Factory : minimum 20 € ; Couscous Atlas : minimum 25 €</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Panier de 13,90 € chez Couscous Atlas ; 3,50 € chez Burger Factory (API)</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>1. Remplir un panier sous le minimum
+2. Aller au checkout
+3. Valider</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Validation refusée avec un message indiquant le minimum</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Commande #19 confirmée à 13,90 € (minimum 25 €) ; via API, commande à 3,50 € acceptée (201) chez Burger Factory</t>
+        </is>
+      </c>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>BUG-11</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>preuves/ui-commande-sous-minimum-couscous-atlas.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>TC-M16</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Règle métier</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Commande sur un restaurant FERMÉ (interface)</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier qu'on ne peut pas commander chez un restaurant affiché « FERMÉ »</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Night Sushi affiché « FERMÉ »</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Sushi épuisé / Late Sushi Box</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>1. Ouvrir le menu de Night Sushi
+2. Ajouter un produit
+3. Passer commande</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Menu inaccessible ou boutons désactivés</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>« Sushi épuisé ajouté au panier. » puis commande acceptée</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>BUG-06</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>preuves/ui-restaurant-ferme-ajout-panier.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>TC-M17</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Règle métier</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Prix du menu = prix facturé</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Vérifier que le prix unitaire ne change pas entre menu et checkout</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Chicken Teriyaki affiché 13,50 €</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Quantité 2</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>1. Noter le prix
+2. Ajouter 2 unités
+3. Vérifier le sous-total au checkout</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Sous-total = 27,00 €</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Sous-total 27,00 €</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Marina</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>Navigateur (constat visuel)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renuméroter les bugs restants
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -1432,7 +1432,7 @@
       </ns0:c>
       <ns0:c r="K15" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-06</ns0:t>
+          <ns0:t>BUG-05</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="L15" s="3" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </ns0:c>
       <ns0:c r="M15" s="3" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-06 (réponse API)</ns0:t>
+          <ns0:t>BUG-05 (réponse API)</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -1499,7 +1499,7 @@
       </ns0:c>
       <ns0:c r="K16" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-07</ns0:t>
+          <ns0:t>BUG-06</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="L16" s="3" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </ns0:c>
       <ns0:c r="M16" s="3" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-07 (réponse API)</ns0:t>
+          <ns0:t>BUG-06 (réponse API)</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -1566,7 +1566,7 @@
       </ns0:c>
       <ns0:c r="K17" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-04</ns0:t>
+          <ns0:t>BUG-03</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="L17" s="3" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </ns0:c>
       <ns0:c r="M17" s="3" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-04 (réponse API)</ns0:t>
+          <ns0:t>BUG-03 (réponse API)</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -1829,7 +1829,7 @@
       </ns0:c>
       <ns0:c r="K21" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-03</ns0:t>
+          <ns0:t>BUG-02</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="L21" s="3" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </ns0:c>
       <ns0:c r="M21" s="3" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-03 (séquence API)</ns0:t>
+          <ns0:t>BUG-02 (séquence API)</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -1898,7 +1898,7 @@
       </ns0:c>
       <ns0:c r="K22" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-05</ns0:t>
+          <ns0:t>BUG-04</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="L22" s="3" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </ns0:c>
       <ns0:c r="M22" s="3" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-05 (compteurs avant/après)</ns0:t>
+          <ns0:t>BUG-04 (compteurs avant/après)</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -1967,7 +1967,7 @@
       </ns0:c>
       <ns0:c r="K23" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-10</ns0:t>
+          <ns0:t>BUG-07</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="L23" s="3" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </ns0:c>
       <ns0:c r="M23" s="3" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-10 (requête SQL)</ns0:t>
+          <ns0:t>BUG-07 (requête SQL)</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -2101,7 +2101,7 @@
       </ns0:c>
       <ns0:c r="K25" s="5" t="inlineStr">
         <ns0:is>
-          <ns0:t>BUG-11</ns0:t>
+          <ns0:t>BUG-08</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="L25" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Remplace Marina par Elodie dans la colonne Testé par
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -931,7 +931,7 @@
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Marina</t>
+          <t>Elodie</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>Marina</t>
+          <t>Elodie</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">

</xml_diff>